<commit_message>
Fascia anteriore in morale 80x80 di coltello
- La fascia anteriore passa da KVH 80x120 di piatto a morale di abete
  80x80 (Tecnomat): gambe anteriori arretrate di 80 come le posteriori,
  traverse laterali 400 invece di 360, 620 mm liberi sotto la fascia.
- Viti 8x160 con sola svasatura anche davanti (niente lamatura e tappi).
- KVH: 4 barre invece di 5. Tavolo base ~591 EUR.
- Modello, fori (0 collisioni), taglio, costi, tavole e manuali rigenerati.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014ifKLy6ksUu35M7vyqXshy
</commit_message>
<xml_diff>
--- a/confronto_prezzi_negozi.xlsx
+++ b/confronto_prezzi_negozi.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="183">
   <si>
     <t xml:space="preserve">Confronto prezzi Tecnomat · OBI · Leroy Merlin (18/10/2026)</t>
   </si>
@@ -324,6 +324,24 @@
   </si>
   <si>
     <t xml:space="preserve">24 viti = 47,88 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fascia anteriore 80×80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Morale abete grezzo 80×80×4000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">80×80×4000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Morale listello travetto piallato 78×78 (MP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">78×78×2000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 mm più piccolo, solo online</t>
   </si>
   <si>
     <t xml:space="preserve">Fascia 2000 (alternativa)</t>
@@ -1016,7 +1034,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -1888,29 +1906,29 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="8" t="s">
+      <c r="A38" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C38" s="9" t="s">
+      <c r="C38" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="D38" s="8" t="s">
+      <c r="D38" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="E38" s="10" t="n">
-        <v>42</v>
-      </c>
-      <c r="F38" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="G38" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="H38" s="9" t="s">
-        <v>104</v>
+      <c r="E38" s="6" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H38" s="5" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1918,33 +1936,31 @@
         <v>101</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C39" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="D39" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="D39" s="8" t="s">
+      <c r="E39" s="10" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="F39" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G39" s="8"/>
+      <c r="H39" s="9" t="s">
         <v>106</v>
-      </c>
-      <c r="E39" s="10" t="n">
-        <v>18</v>
-      </c>
-      <c r="F39" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="G39" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="H39" s="9" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="8" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C40" s="9" t="s">
         <v>108</v>
@@ -1953,7 +1969,7 @@
         <v>109</v>
       </c>
       <c r="E40" s="10" t="n">
-        <v>48.99</v>
+        <v>42</v>
       </c>
       <c r="F40" s="8" t="s">
         <v>14</v>
@@ -1966,34 +1982,34 @@
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="4" t="s">
+      <c r="A41" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C41" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="B41" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C41" s="5" t="s">
+      <c r="D41" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="D41" s="4" t="s">
+      <c r="E41" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G41" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H41" s="9" t="s">
         <v>113</v>
-      </c>
-      <c r="E41" s="6" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="F41" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G41" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="H41" s="5" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="8" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B42" s="8" t="s">
         <v>18</v>
@@ -2002,84 +2018,86 @@
         <v>114</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E42" s="10" t="n">
+        <v>48.99</v>
+      </c>
+      <c r="F42" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G42" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H42" s="9" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E43" s="6" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G43" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H43" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="D44" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="E44" s="10" t="n">
         <v>1.75</v>
       </c>
-      <c r="F42" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="G42" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="H42" s="9"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="B43" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C43" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="D43" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="E43" s="10" t="n">
-        <v>3.19</v>
-      </c>
-      <c r="F43" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="G43" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="H43" s="9"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C44" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="D44" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="E44" s="6" t="n">
-        <v>3.69</v>
-      </c>
-      <c r="F44" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="G44" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="H44" s="5" t="s">
-        <v>16</v>
-      </c>
+      <c r="F44" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G44" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H44" s="9"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="C45" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="D45" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="D45" s="8" t="s">
-        <v>120</v>
-      </c>
       <c r="E45" s="10" t="n">
-        <v>0.8</v>
+        <v>3.19</v>
       </c>
       <c r="F45" s="8" t="s">
         <v>14</v>
@@ -2087,16 +2105,14 @@
       <c r="G45" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="H45" s="9" t="s">
-        <v>121</v>
-      </c>
+      <c r="H45" s="9"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
         <v>122</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="C46" s="5" t="s">
         <v>123</v>
@@ -2105,10 +2121,10 @@
         <v>124</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>10.9</v>
+        <v>3.69</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>125</v>
+        <v>86</v>
       </c>
       <c r="G46" s="7" t="s">
         <v>15</v>
@@ -2122,119 +2138,119 @@
         <v>122</v>
       </c>
       <c r="B47" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C47" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="D47" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="E47" s="10" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F47" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G47" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H47" s="9" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="E48" s="6" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="G48" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H48" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="B49" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C47" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="D47" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="E47" s="10" t="n">
+      <c r="C49" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="D49" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="E49" s="10" t="n">
         <v>10.9</v>
       </c>
-      <c r="F47" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="G47" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="H47" s="9"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="B48" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C48" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="D48" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="E48" s="10" t="n">
-        <v>37.99</v>
-      </c>
-      <c r="F48" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="G48" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="H48" s="9"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="B49" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C49" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="E49" s="6" t="n">
-        <v>2.89</v>
-      </c>
-      <c r="F49" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G49" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="H49" s="5" t="s">
-        <v>16</v>
-      </c>
+      <c r="F49" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="G49" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H49" s="9"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="C50" s="9" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E50" s="10" t="n">
-        <v>0.8</v>
+        <v>37.99</v>
       </c>
       <c r="F50" s="8" t="s">
-        <v>14</v>
+        <v>133</v>
       </c>
       <c r="G50" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="H50" s="9" t="s">
-        <v>133</v>
-      </c>
+      <c r="H50" s="9"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E51" s="6" t="n">
-        <v>1.05</v>
+        <v>2.89</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>99</v>
+        <v>14</v>
       </c>
       <c r="G51" s="7" t="s">
         <v>15</v>
@@ -2245,19 +2261,19 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C52" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="D52" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="D52" s="8" t="s">
-        <v>136</v>
-      </c>
       <c r="E52" s="10" t="n">
-        <v>0.99</v>
+        <v>0.8</v>
       </c>
       <c r="F52" s="8" t="s">
         <v>14</v>
@@ -2265,63 +2281,115 @@
       <c r="G52" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="H52" s="9"/>
+      <c r="H52" s="9" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>11</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E53" s="6" t="n">
-        <v>8.55</v>
+        <v>1.05</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>14</v>
+        <v>99</v>
       </c>
       <c r="G53" s="7" t="s">
         <v>15</v>
       </c>
       <c r="H53" s="5" t="s">
-        <v>141</v>
+        <v>16</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="8" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B54" s="8" t="s">
         <v>18</v>
       </c>
       <c r="C54" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="D54" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="D54" s="8" t="s">
-        <v>143</v>
-      </c>
       <c r="E54" s="10" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="F54" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G54" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H54" s="9"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C55" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="E55" s="6" t="n">
+        <v>8.55</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G55" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H55" s="5" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C56" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="D56" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="E56" s="10" t="n">
         <v>36.95</v>
       </c>
-      <c r="F54" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="G54" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="H54" s="9" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="2" t="s">
-        <v>145</v>
+      <c r="F56" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G56" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H56" s="9" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="2" t="s">
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -2360,22 +2428,23 @@
     <hyperlink ref="G36" r:id="rId32" display="apri"/>
     <hyperlink ref="G37" r:id="rId33" display="apri"/>
     <hyperlink ref="G38" r:id="rId34" display="apri"/>
-    <hyperlink ref="G39" r:id="rId35" display="apri"/>
-    <hyperlink ref="G40" r:id="rId36" display="apri"/>
-    <hyperlink ref="G41" r:id="rId37" display="apri"/>
-    <hyperlink ref="G42" r:id="rId38" display="apri"/>
-    <hyperlink ref="G43" r:id="rId39" display="apri"/>
-    <hyperlink ref="G44" r:id="rId40" display="apri"/>
-    <hyperlink ref="G45" r:id="rId41" display="apri"/>
-    <hyperlink ref="G46" r:id="rId42" display="apri"/>
-    <hyperlink ref="G47" r:id="rId43" display="apri"/>
-    <hyperlink ref="G48" r:id="rId44" display="apri"/>
-    <hyperlink ref="G49" r:id="rId45" display="apri"/>
-    <hyperlink ref="G50" r:id="rId46" display="apri"/>
-    <hyperlink ref="G51" r:id="rId47" display="apri"/>
-    <hyperlink ref="G52" r:id="rId48" display="apri"/>
-    <hyperlink ref="G53" r:id="rId49" display="apri"/>
-    <hyperlink ref="G54" r:id="rId50" display="apri"/>
+    <hyperlink ref="G40" r:id="rId35" display="apri"/>
+    <hyperlink ref="G41" r:id="rId36" display="apri"/>
+    <hyperlink ref="G42" r:id="rId37" display="apri"/>
+    <hyperlink ref="G43" r:id="rId38" display="apri"/>
+    <hyperlink ref="G44" r:id="rId39" display="apri"/>
+    <hyperlink ref="G45" r:id="rId40" display="apri"/>
+    <hyperlink ref="G46" r:id="rId41" display="apri"/>
+    <hyperlink ref="G47" r:id="rId42" display="apri"/>
+    <hyperlink ref="G48" r:id="rId43" display="apri"/>
+    <hyperlink ref="G49" r:id="rId44" display="apri"/>
+    <hyperlink ref="G50" r:id="rId45" display="apri"/>
+    <hyperlink ref="G51" r:id="rId46" display="apri"/>
+    <hyperlink ref="G52" r:id="rId47" display="apri"/>
+    <hyperlink ref="G53" r:id="rId48" display="apri"/>
+    <hyperlink ref="G54" r:id="rId49" display="apri"/>
+    <hyperlink ref="G55" r:id="rId50" display="apri"/>
+    <hyperlink ref="G56" r:id="rId51" display="apri"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2406,27 +2475,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>9</v>
@@ -2434,10 +2503,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>22</v>
@@ -2453,15 +2522,15 @@
         <v>22.24</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>22</v>
@@ -2480,13 +2549,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="D6" s="12" t="n">
         <v>38</v>
@@ -2499,15 +2568,15 @@
         <v>30.4</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>11</v>
@@ -2526,10 +2595,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>22</v>
@@ -2548,10 +2617,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>11</v>
@@ -2567,15 +2636,15 @@
         <v>41.9</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="C10" s="8" t="s">
         <v>22</v>
@@ -2591,15 +2660,15 @@
         <v>11.07</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>22</v>
@@ -2615,15 +2684,15 @@
         <v>119.96</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>11</v>
@@ -2642,10 +2711,10 @@
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>22</v>
@@ -2661,18 +2730,18 @@
         <v>27.8</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="D14" s="12" t="n">
         <v>20</v>
@@ -2685,15 +2754,15 @@
         <v>16</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>11</v>
@@ -2709,15 +2778,15 @@
         <v>27.45</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>22</v>
@@ -2736,7 +2805,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E18" s="14" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="F18" s="15" t="n">
         <f aca="false">SUMIFS(F4:F16,A4:A16,"A · Bulloni + dadi a tamburo (precedente)")</f>
@@ -2745,7 +2814,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E19" s="14" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="F19" s="15" t="n">
         <f aca="false">SUMIFS(F4:F16,A4:A16,"B · Viti strutturali")</f>
@@ -2754,7 +2823,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E20" s="14" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="F20" s="15" t="n">
         <f aca="false">SUMIFS(F4:F16,A4:A16,"C · Staffe metalliche")</f>
@@ -2763,7 +2832,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E21" s="14" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="F21" s="15" t="n">
         <f aca="false">SUMIFS(F4:F16,A4:A16,"D · Telai + fasce (adottata)")</f>

</xml_diff>